<commit_message>
lastest changes and Rahul shetty was deleted
</commit_message>
<xml_diff>
--- a/001EffortTracker/KT Plan.xlsx
+++ b/001EffortTracker/KT Plan.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="688" uniqueCount="363">
   <si>
     <t>Playwright: Web Automation Testing From Zero to Hero - Artem Bondar</t>
   </si>
@@ -1120,7 +1120,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1178,12 +1178,6 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1232,7 +1226,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="51">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1380,15 +1374,6 @@
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1701,7 +1686,7 @@
     <col min="1" max="1" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="53" width="6.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="50" width="6.719285714285714" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="47" width="38.86214285714286" customWidth="1" bestFit="1"/>
     <col min="6" max="6" style="23" width="7.719285714285714" customWidth="1" bestFit="1"/>
     <col min="7" max="7" style="47" width="23.862142857142857" customWidth="1" bestFit="1"/>
@@ -2246,61 +2231,61 @@
       <c r="A30" s="22"/>
       <c r="B30" s="22"/>
       <c r="C30" s="22"/>
-      <c r="D30" s="50"/>
-      <c r="E30" s="51"/>
-      <c r="F30" s="52"/>
-      <c r="G30" s="51"/>
-      <c r="H30" s="51"/>
+      <c r="D30" s="48"/>
+      <c r="E30" s="35"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="35"/>
+      <c r="H30" s="35"/>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
       <c r="A31" s="22"/>
       <c r="B31" s="22"/>
       <c r="C31" s="22"/>
-      <c r="D31" s="50"/>
-      <c r="E31" s="51"/>
-      <c r="F31" s="52"/>
-      <c r="G31" s="51"/>
-      <c r="H31" s="51"/>
+      <c r="D31" s="48"/>
+      <c r="E31" s="35"/>
+      <c r="F31" s="21"/>
+      <c r="G31" s="35"/>
+      <c r="H31" s="35"/>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
       <c r="A32" s="22"/>
       <c r="B32" s="22"/>
       <c r="C32" s="22"/>
-      <c r="D32" s="50"/>
-      <c r="E32" s="51"/>
-      <c r="F32" s="52"/>
-      <c r="G32" s="51"/>
-      <c r="H32" s="51"/>
+      <c r="D32" s="48"/>
+      <c r="E32" s="35"/>
+      <c r="F32" s="21"/>
+      <c r="G32" s="35"/>
+      <c r="H32" s="35"/>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
       <c r="A33" s="22"/>
       <c r="B33" s="22"/>
       <c r="C33" s="22"/>
-      <c r="D33" s="50"/>
-      <c r="E33" s="51"/>
-      <c r="F33" s="52"/>
-      <c r="G33" s="51"/>
-      <c r="H33" s="51"/>
+      <c r="D33" s="48"/>
+      <c r="E33" s="35"/>
+      <c r="F33" s="21"/>
+      <c r="G33" s="35"/>
+      <c r="H33" s="35"/>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
       <c r="A34" s="22"/>
       <c r="B34" s="22"/>
       <c r="C34" s="22"/>
-      <c r="D34" s="50"/>
-      <c r="E34" s="51"/>
-      <c r="F34" s="52"/>
-      <c r="G34" s="51"/>
-      <c r="H34" s="51"/>
+      <c r="D34" s="48"/>
+      <c r="E34" s="35"/>
+      <c r="F34" s="21"/>
+      <c r="G34" s="35"/>
+      <c r="H34" s="35"/>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
       <c r="A35" s="22"/>
       <c r="B35" s="22"/>
       <c r="C35" s="22"/>
-      <c r="D35" s="50"/>
-      <c r="E35" s="51"/>
-      <c r="F35" s="52"/>
-      <c r="G35" s="51"/>
-      <c r="H35" s="51"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="35"/>
+      <c r="F35" s="21"/>
+      <c r="G35" s="35"/>
+      <c r="H35" s="35"/>
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
       <c r="A36" s="22"/>
@@ -3946,7 +3931,9 @@
         <v>276</v>
       </c>
       <c r="F74" s="2"/>
-      <c r="G74" s="17"/>
+      <c r="G74" s="17" t="s">
+        <v>198</v>
+      </c>
       <c r="H74" s="17"/>
       <c r="I74" s="35"/>
     </row>
@@ -3967,7 +3954,9 @@
         <v>280</v>
       </c>
       <c r="F75" s="2"/>
-      <c r="G75" s="17"/>
+      <c r="G75" s="17" t="s">
+        <v>198</v>
+      </c>
       <c r="H75" s="17"/>
       <c r="I75" s="35"/>
     </row>
@@ -3988,7 +3977,9 @@
         <v>280</v>
       </c>
       <c r="F76" s="2"/>
-      <c r="G76" s="17"/>
+      <c r="G76" s="17" t="s">
+        <v>198</v>
+      </c>
       <c r="H76" s="17"/>
       <c r="I76" s="35"/>
     </row>
@@ -4051,7 +4042,7 @@
         <v>282</v>
       </c>
       <c r="C80" s="44">
-        <v>28.118275462962963</v>
+        <v>29.118159722222224</v>
       </c>
       <c r="D80" s="18">
         <v>45374</v>
@@ -4072,7 +4063,7 @@
         <v>282</v>
       </c>
       <c r="C81" s="44">
-        <v>28.118275462962963</v>
+        <v>29.118159722222224</v>
       </c>
       <c r="D81" s="18">
         <v>45375</v>
@@ -4093,7 +4084,7 @@
         <v>282</v>
       </c>
       <c r="C82" s="44">
-        <v>28.118275462962963</v>
+        <v>29.118159722222224</v>
       </c>
       <c r="D82" s="18">
         <v>45376</v>
@@ -4114,7 +4105,7 @@
         <v>282</v>
       </c>
       <c r="C83" s="44">
-        <v>28.118275462962963</v>
+        <v>29.118159722222224</v>
       </c>
       <c r="D83" s="18">
         <v>45377</v>

</xml_diff>

<commit_message>
new day new concepts
</commit_message>
<xml_diff>
--- a/001EffortTracker/KT Plan.xlsx
+++ b/001EffortTracker/KT Plan.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="363">
   <si>
     <t>Playwright: Web Automation Testing From Zero to Hero - Artem Bondar</t>
   </si>
@@ -1120,7 +1120,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1168,12 +1168,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1232,7 +1226,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="52">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1330,9 +1324,6 @@
     <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1341,9 +1332,6 @@
     </xf>
     <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1387,7 +1375,7 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -1701,11 +1689,11 @@
     <col min="1" max="1" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="53" width="6.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="50" width="38.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="51" width="6.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="48" width="38.86214285714286" customWidth="1" bestFit="1"/>
     <col min="6" max="6" style="23" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="50" width="23.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="50" width="41.29071428571429" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="48" width="23.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="48" width="41.29071428571429" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -1713,10 +1701,10 @@
       <c r="B1" s="22"/>
       <c r="C1" s="22"/>
       <c r="D1" s="21"/>
-      <c r="E1" s="38"/>
+      <c r="E1" s="36"/>
       <c r="F1" s="21"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="22"/>
@@ -1728,7 +1716,7 @@
       <c r="E2" s="14" t="s">
         <v>319</v>
       </c>
-      <c r="F2" s="51" t="s">
+      <c r="F2" s="49" t="s">
         <v>320</v>
       </c>
       <c r="G2" s="14" t="s">
@@ -1828,7 +1816,7 @@
       <c r="G7" s="17" t="s">
         <v>327</v>
       </c>
-      <c r="H7" s="52" t="s">
+      <c r="H7" s="50" t="s">
         <v>329</v>
       </c>
     </row>
@@ -1974,7 +1962,7 @@
       <c r="G15" s="17" t="s">
         <v>339</v>
       </c>
-      <c r="H15" s="52" t="s">
+      <c r="H15" s="50" t="s">
         <v>340</v>
       </c>
     </row>
@@ -1994,7 +1982,7 @@
       <c r="G16" s="17" t="s">
         <v>339</v>
       </c>
-      <c r="H16" s="52" t="s">
+      <c r="H16" s="50" t="s">
         <v>342</v>
       </c>
     </row>
@@ -2014,7 +2002,7 @@
       <c r="G17" s="17" t="s">
         <v>339</v>
       </c>
-      <c r="H17" s="52" t="s">
+      <c r="H17" s="50" t="s">
         <v>344</v>
       </c>
     </row>
@@ -2049,82 +2037,82 @@
       <c r="F19" s="21">
         <v>1</v>
       </c>
-      <c r="G19" s="38" t="s">
+      <c r="G19" s="36" t="s">
         <v>327</v>
       </c>
-      <c r="H19" s="38"/>
+      <c r="H19" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
       <c r="A20" s="22"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
-      <c r="D20" s="51">
+      <c r="D20" s="49">
         <v>18</v>
       </c>
-      <c r="E20" s="38" t="s">
+      <c r="E20" s="36" t="s">
         <v>347</v>
       </c>
       <c r="F20" s="21">
         <v>2</v>
       </c>
-      <c r="G20" s="38" t="s">
+      <c r="G20" s="36" t="s">
         <v>327</v>
       </c>
-      <c r="H20" s="38"/>
+      <c r="H20" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="22"/>
       <c r="B21" s="22"/>
       <c r="C21" s="22"/>
-      <c r="D21" s="51">
+      <c r="D21" s="49">
         <v>19</v>
       </c>
-      <c r="E21" s="38" t="s">
+      <c r="E21" s="36" t="s">
         <v>348</v>
       </c>
       <c r="F21" s="21">
         <v>1</v>
       </c>
-      <c r="G21" s="38" t="s">
+      <c r="G21" s="36" t="s">
         <v>327</v>
       </c>
-      <c r="H21" s="38"/>
+      <c r="H21" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
       <c r="A22" s="22"/>
       <c r="B22" s="22"/>
       <c r="C22" s="22"/>
-      <c r="D22" s="51">
+      <c r="D22" s="49">
         <v>20</v>
       </c>
-      <c r="E22" s="38" t="s">
+      <c r="E22" s="36" t="s">
         <v>349</v>
       </c>
       <c r="F22" s="21">
         <v>1</v>
       </c>
-      <c r="G22" s="38" t="s">
+      <c r="G22" s="36" t="s">
         <v>327</v>
       </c>
-      <c r="H22" s="38"/>
+      <c r="H22" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
       <c r="A23" s="22"/>
       <c r="B23" s="22"/>
       <c r="C23" s="22"/>
-      <c r="D23" s="51">
+      <c r="D23" s="49">
         <v>21</v>
       </c>
-      <c r="E23" s="38" t="s">
+      <c r="E23" s="36" t="s">
         <v>350</v>
       </c>
       <c r="F23" s="21">
         <v>1</v>
       </c>
-      <c r="G23" s="38" t="s">
+      <c r="G23" s="36" t="s">
         <v>351</v>
       </c>
-      <c r="H23" s="38" t="s">
+      <c r="H23" s="36" t="s">
         <v>352</v>
       </c>
     </row>
@@ -2132,19 +2120,19 @@
       <c r="A24" s="22"/>
       <c r="B24" s="22"/>
       <c r="C24" s="22"/>
-      <c r="D24" s="51">
+      <c r="D24" s="49">
         <v>22</v>
       </c>
-      <c r="E24" s="38" t="s">
+      <c r="E24" s="36" t="s">
         <v>353</v>
       </c>
       <c r="F24" s="21">
         <v>1</v>
       </c>
-      <c r="G24" s="38" t="s">
+      <c r="G24" s="36" t="s">
         <v>331</v>
       </c>
-      <c r="H24" s="38" t="s">
+      <c r="H24" s="36" t="s">
         <v>354</v>
       </c>
     </row>
@@ -2152,35 +2140,35 @@
       <c r="A25" s="22"/>
       <c r="B25" s="22"/>
       <c r="C25" s="22"/>
-      <c r="D25" s="51">
+      <c r="D25" s="49">
         <v>23</v>
       </c>
-      <c r="E25" s="38" t="s">
+      <c r="E25" s="36" t="s">
         <v>355</v>
       </c>
       <c r="F25" s="21">
         <v>1</v>
       </c>
-      <c r="G25" s="38" t="s">
+      <c r="G25" s="36" t="s">
         <v>327</v>
       </c>
-      <c r="H25" s="38"/>
+      <c r="H25" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5">
       <c r="A26" s="22"/>
       <c r="B26" s="22"/>
       <c r="C26" s="22"/>
-      <c r="D26" s="51">
+      <c r="D26" s="49">
         <v>24</v>
       </c>
-      <c r="E26" s="38" t="s">
+      <c r="E26" s="36" t="s">
         <v>356</v>
       </c>
       <c r="F26" s="21">
         <v>1</v>
       </c>
-      <c r="G26" s="38"/>
-      <c r="H26" s="38"/>
+      <c r="G26" s="36"/>
+      <c r="H26" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="20.25">
       <c r="A27" s="22"/>
@@ -2195,7 +2183,7 @@
       <c r="F27" s="21">
         <v>1</v>
       </c>
-      <c r="G27" s="38" t="s">
+      <c r="G27" s="36" t="s">
         <v>331</v>
       </c>
       <c r="H27" s="17" t="s">
@@ -2206,19 +2194,19 @@
       <c r="A28" s="22"/>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
-      <c r="D28" s="51">
+      <c r="D28" s="49">
         <v>26</v>
       </c>
-      <c r="E28" s="38" t="s">
+      <c r="E28" s="36" t="s">
         <v>359</v>
       </c>
       <c r="F28" s="21">
         <v>1</v>
       </c>
-      <c r="G28" s="38" t="s">
+      <c r="G28" s="36" t="s">
         <v>339</v>
       </c>
-      <c r="H28" s="38" t="s">
+      <c r="H28" s="36" t="s">
         <v>360</v>
       </c>
     </row>
@@ -2226,19 +2214,19 @@
       <c r="A29" s="22"/>
       <c r="B29" s="22"/>
       <c r="C29" s="22"/>
-      <c r="D29" s="51">
+      <c r="D29" s="49">
         <v>27</v>
       </c>
-      <c r="E29" s="38" t="s">
+      <c r="E29" s="36" t="s">
         <v>361</v>
       </c>
       <c r="F29" s="21">
         <v>1</v>
       </c>
-      <c r="G29" s="38" t="s">
+      <c r="G29" s="36" t="s">
         <v>339</v>
       </c>
-      <c r="H29" s="38" t="s">
+      <c r="H29" s="36" t="s">
         <v>362</v>
       </c>
     </row>
@@ -2246,61 +2234,61 @@
       <c r="A30" s="22"/>
       <c r="B30" s="22"/>
       <c r="C30" s="22"/>
-      <c r="D30" s="51"/>
-      <c r="E30" s="38"/>
+      <c r="D30" s="49"/>
+      <c r="E30" s="36"/>
       <c r="F30" s="21"/>
-      <c r="G30" s="38"/>
-      <c r="H30" s="38"/>
+      <c r="G30" s="36"/>
+      <c r="H30" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="19.5">
       <c r="A31" s="22"/>
       <c r="B31" s="22"/>
       <c r="C31" s="22"/>
-      <c r="D31" s="51"/>
-      <c r="E31" s="38"/>
+      <c r="D31" s="49"/>
+      <c r="E31" s="36"/>
       <c r="F31" s="21"/>
-      <c r="G31" s="38"/>
-      <c r="H31" s="38"/>
+      <c r="G31" s="36"/>
+      <c r="H31" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="19.5">
       <c r="A32" s="22"/>
       <c r="B32" s="22"/>
       <c r="C32" s="22"/>
-      <c r="D32" s="51"/>
-      <c r="E32" s="38"/>
+      <c r="D32" s="49"/>
+      <c r="E32" s="36"/>
       <c r="F32" s="21"/>
-      <c r="G32" s="38"/>
-      <c r="H32" s="38"/>
+      <c r="G32" s="36"/>
+      <c r="H32" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="19.5">
       <c r="A33" s="22"/>
       <c r="B33" s="22"/>
       <c r="C33" s="22"/>
-      <c r="D33" s="51"/>
-      <c r="E33" s="38"/>
+      <c r="D33" s="49"/>
+      <c r="E33" s="36"/>
       <c r="F33" s="21"/>
-      <c r="G33" s="38"/>
-      <c r="H33" s="38"/>
+      <c r="G33" s="36"/>
+      <c r="H33" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="19.5">
       <c r="A34" s="22"/>
       <c r="B34" s="22"/>
       <c r="C34" s="22"/>
-      <c r="D34" s="51"/>
-      <c r="E34" s="38"/>
+      <c r="D34" s="49"/>
+      <c r="E34" s="36"/>
       <c r="F34" s="21"/>
-      <c r="G34" s="38"/>
-      <c r="H34" s="38"/>
+      <c r="G34" s="36"/>
+      <c r="H34" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="19.5">
       <c r="A35" s="22"/>
       <c r="B35" s="22"/>
       <c r="C35" s="22"/>
-      <c r="D35" s="51"/>
-      <c r="E35" s="38"/>
+      <c r="D35" s="49"/>
+      <c r="E35" s="36"/>
       <c r="F35" s="21"/>
-      <c r="G35" s="38"/>
-      <c r="H35" s="38"/>
+      <c r="G35" s="36"/>
+      <c r="H35" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="20.25">
       <c r="A36" s="22"/>
@@ -2309,7 +2297,7 @@
       <c r="D36" s="20"/>
       <c r="E36" s="17"/>
       <c r="F36" s="21"/>
-      <c r="G36" s="38"/>
+      <c r="G36" s="36"/>
       <c r="H36" s="17"/>
     </row>
   </sheetData>
@@ -2326,97 +2314,97 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="23" width="7.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="50" width="60.29071428571429" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="35" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="36" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="48" width="60.29071428571429" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="34" width="10.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="35" width="7.719285714285714" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="6" max="6" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="50" width="12.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="50" width="15.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="50" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="48" width="12.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="48" width="15.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="48" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="21"/>
-      <c r="B1" s="38" t="s">
+      <c r="B1" s="36" t="s">
         <v>191</v>
       </c>
       <c r="C1" s="31"/>
       <c r="D1" s="32"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="47.25">
       <c r="A2" s="21">
         <v>1</v>
       </c>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="36" t="s">
         <v>192</v>
       </c>
       <c r="C2" s="31"/>
       <c r="D2" s="32"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="38"/>
-      <c r="H2" s="38"/>
-      <c r="I2" s="38"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="21">
         <v>2</v>
       </c>
-      <c r="B3" s="38" t="s">
+      <c r="B3" s="36" t="s">
         <v>193</v>
       </c>
       <c r="C3" s="31"/>
       <c r="D3" s="32"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="38"/>
-      <c r="H3" s="38"/>
-      <c r="I3" s="38"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="21">
         <v>3</v>
       </c>
-      <c r="B4" s="38" t="s">
+      <c r="B4" s="36" t="s">
         <v>194</v>
       </c>
       <c r="C4" s="31"/>
       <c r="D4" s="32"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
-      <c r="G4" s="38"/>
-      <c r="H4" s="38"/>
-      <c r="I4" s="38"/>
+      <c r="G4" s="36"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="21"/>
-      <c r="B5" s="38"/>
+      <c r="B5" s="36"/>
       <c r="C5" s="31"/>
       <c r="D5" s="32"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
-      <c r="G5" s="38"/>
-      <c r="H5" s="38"/>
-      <c r="I5" s="38"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="36"/>
+      <c r="I5" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
-      <c r="A6" s="39" t="s">
+      <c r="A6" s="37" t="s">
         <v>195</v>
       </c>
-      <c r="B6" s="40"/>
-      <c r="C6" s="41"/>
-      <c r="D6" s="42"/>
+      <c r="B6" s="38"/>
+      <c r="C6" s="39"/>
+      <c r="D6" s="40"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="38"/>
+      <c r="G6" s="38"/>
+      <c r="H6" s="38"/>
+      <c r="I6" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="13" t="s">
@@ -2443,7 +2431,7 @@
       <c r="H7" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="I7" s="38"/>
+      <c r="I7" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="33.75">
       <c r="A8" s="15">
@@ -2466,7 +2454,7 @@
         <v>16</v>
       </c>
       <c r="H8" s="17"/>
-      <c r="I8" s="38"/>
+      <c r="I8" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="15">
@@ -2489,7 +2477,7 @@
         <v>16</v>
       </c>
       <c r="H9" s="17"/>
-      <c r="I9" s="38"/>
+      <c r="I9" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="15">
@@ -2512,7 +2500,7 @@
         <v>16</v>
       </c>
       <c r="H10" s="17"/>
-      <c r="I10" s="43" t="s">
+      <c r="I10" s="41" t="s">
         <v>201</v>
       </c>
     </row>
@@ -2537,7 +2525,7 @@
         <v>16</v>
       </c>
       <c r="H11" s="17"/>
-      <c r="I11" s="38"/>
+      <c r="I11" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="15">
@@ -2560,7 +2548,7 @@
         <v>16</v>
       </c>
       <c r="H12" s="17"/>
-      <c r="I12" s="38"/>
+      <c r="I12" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="15">
@@ -2583,7 +2571,7 @@
         <v>16</v>
       </c>
       <c r="H13" s="17"/>
-      <c r="I13" s="38"/>
+      <c r="I13" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="15">
@@ -2606,7 +2594,7 @@
         <v>16</v>
       </c>
       <c r="H14" s="17"/>
-      <c r="I14" s="38"/>
+      <c r="I14" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="15">
@@ -2629,7 +2617,7 @@
         <v>16</v>
       </c>
       <c r="H15" s="17"/>
-      <c r="I15" s="38"/>
+      <c r="I15" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="15">
@@ -2652,7 +2640,7 @@
         <v>16</v>
       </c>
       <c r="H16" s="17"/>
-      <c r="I16" s="38"/>
+      <c r="I16" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="15">
@@ -2675,7 +2663,7 @@
         <v>16</v>
       </c>
       <c r="H17" s="17"/>
-      <c r="I17" s="38"/>
+      <c r="I17" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
       <c r="A18" s="15">
@@ -2698,7 +2686,7 @@
         <v>16</v>
       </c>
       <c r="H18" s="17"/>
-      <c r="I18" s="38"/>
+      <c r="I18" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="15">
@@ -2721,7 +2709,7 @@
         <v>16</v>
       </c>
       <c r="H19" s="17"/>
-      <c r="I19" s="38"/>
+      <c r="I19" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="33.75">
       <c r="A20" s="15">
@@ -2744,7 +2732,7 @@
         <v>16</v>
       </c>
       <c r="H20" s="17"/>
-      <c r="I20" s="38"/>
+      <c r="I20" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="15">
@@ -2767,7 +2755,7 @@
         <v>16</v>
       </c>
       <c r="H21" s="17"/>
-      <c r="I21" s="38"/>
+      <c r="I21" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
       <c r="A22" s="15">
@@ -2790,7 +2778,7 @@
         <v>16</v>
       </c>
       <c r="H22" s="17"/>
-      <c r="I22" s="38"/>
+      <c r="I22" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
       <c r="A23" s="15">
@@ -2813,7 +2801,7 @@
         <v>16</v>
       </c>
       <c r="H23" s="17"/>
-      <c r="I23" s="38"/>
+      <c r="I23" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5">
       <c r="A24" s="15">
@@ -2836,7 +2824,7 @@
         <v>16</v>
       </c>
       <c r="H24" s="17"/>
-      <c r="I24" s="38"/>
+      <c r="I24" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="19.5">
       <c r="A25" s="15">
@@ -2859,7 +2847,7 @@
         <v>16</v>
       </c>
       <c r="H25" s="17"/>
-      <c r="I25" s="38"/>
+      <c r="I25" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5">
       <c r="A26" s="15">
@@ -2882,7 +2870,7 @@
         <v>16</v>
       </c>
       <c r="H26" s="17"/>
-      <c r="I26" s="38"/>
+      <c r="I26" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="33.75">
       <c r="A27" s="15">
@@ -2905,7 +2893,7 @@
         <v>16</v>
       </c>
       <c r="H27" s="17"/>
-      <c r="I27" s="38"/>
+      <c r="I27" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="19.5">
       <c r="A28" s="15">
@@ -2928,7 +2916,7 @@
         <v>16</v>
       </c>
       <c r="H28" s="17"/>
-      <c r="I28" s="38"/>
+      <c r="I28" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="19.5">
       <c r="A29" s="15">
@@ -2951,7 +2939,7 @@
         <v>16</v>
       </c>
       <c r="H29" s="17"/>
-      <c r="I29" s="38"/>
+      <c r="I29" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="19.5">
       <c r="A30" s="15">
@@ -2974,7 +2962,7 @@
         <v>16</v>
       </c>
       <c r="H30" s="17"/>
-      <c r="I30" s="38"/>
+      <c r="I30" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="19.5">
       <c r="A31" s="15">
@@ -2997,7 +2985,7 @@
         <v>16</v>
       </c>
       <c r="H31" s="17"/>
-      <c r="I31" s="38"/>
+      <c r="I31" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="19.5">
       <c r="A32" s="15">
@@ -3020,7 +3008,7 @@
         <v>16</v>
       </c>
       <c r="H32" s="17"/>
-      <c r="I32" s="38"/>
+      <c r="I32" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="19.5">
       <c r="A33" s="15">
@@ -3043,7 +3031,7 @@
         <v>16</v>
       </c>
       <c r="H33" s="17"/>
-      <c r="I33" s="38"/>
+      <c r="I33" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="19.5">
       <c r="A34" s="15">
@@ -3066,7 +3054,7 @@
         <v>16</v>
       </c>
       <c r="H34" s="17"/>
-      <c r="I34" s="38"/>
+      <c r="I34" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="33.75">
       <c r="A35" s="15">
@@ -3089,7 +3077,7 @@
         <v>16</v>
       </c>
       <c r="H35" s="17"/>
-      <c r="I35" s="38"/>
+      <c r="I35" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="19.5">
       <c r="A36" s="15">
@@ -3112,7 +3100,7 @@
         <v>16</v>
       </c>
       <c r="H36" s="17"/>
-      <c r="I36" s="38"/>
+      <c r="I36" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="19.5">
       <c r="A37" s="15">
@@ -3135,7 +3123,7 @@
         <v>16</v>
       </c>
       <c r="H37" s="17"/>
-      <c r="I37" s="38"/>
+      <c r="I37" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="19.5">
       <c r="A38" s="15">
@@ -3158,7 +3146,7 @@
         <v>16</v>
       </c>
       <c r="H38" s="17"/>
-      <c r="I38" s="38"/>
+      <c r="I38" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="33.75">
       <c r="A39" s="15">
@@ -3181,7 +3169,7 @@
         <v>16</v>
       </c>
       <c r="H39" s="17"/>
-      <c r="I39" s="38"/>
+      <c r="I39" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="19.5">
       <c r="A40" s="15">
@@ -3204,7 +3192,7 @@
         <v>16</v>
       </c>
       <c r="H40" s="17"/>
-      <c r="I40" s="38"/>
+      <c r="I40" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="19.5">
       <c r="A41" s="15">
@@ -3227,7 +3215,7 @@
         <v>16</v>
       </c>
       <c r="H41" s="17"/>
-      <c r="I41" s="38"/>
+      <c r="I41" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="19.5">
       <c r="A42" s="15">
@@ -3250,7 +3238,7 @@
         <v>16</v>
       </c>
       <c r="H42" s="17"/>
-      <c r="I42" s="38"/>
+      <c r="I42" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="19.5">
       <c r="A43" s="15">
@@ -3273,7 +3261,7 @@
         <v>16</v>
       </c>
       <c r="H43" s="17"/>
-      <c r="I43" s="38"/>
+      <c r="I43" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="20.25">
       <c r="A44" s="15">
@@ -3296,18 +3284,18 @@
         <v>16</v>
       </c>
       <c r="H44" s="17"/>
-      <c r="I44" s="38"/>
+      <c r="I44" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="19.5">
       <c r="A45" s="21"/>
-      <c r="B45" s="38"/>
+      <c r="B45" s="36"/>
       <c r="C45" s="31"/>
       <c r="D45" s="32"/>
       <c r="E45" s="2"/>
       <c r="F45" s="2"/>
-      <c r="G45" s="38"/>
-      <c r="H45" s="38"/>
-      <c r="I45" s="38"/>
+      <c r="G45" s="36"/>
+      <c r="H45" s="36"/>
+      <c r="I45" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A46" s="11" t="s">
@@ -3347,7 +3335,7 @@
       <c r="H47" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="I47" s="38"/>
+      <c r="I47" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="33.75">
       <c r="A48" s="15">
@@ -3370,7 +3358,7 @@
         <v>16</v>
       </c>
       <c r="H48" s="17"/>
-      <c r="I48" s="38"/>
+      <c r="I48" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="19.5">
       <c r="A49" s="15">
@@ -3393,7 +3381,7 @@
         <v>16</v>
       </c>
       <c r="H49" s="17"/>
-      <c r="I49" s="38"/>
+      <c r="I49" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="19.5">
       <c r="A50" s="15">
@@ -3416,7 +3404,7 @@
         <v>16</v>
       </c>
       <c r="H50" s="17"/>
-      <c r="I50" s="38"/>
+      <c r="I50" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="19.5">
       <c r="A51" s="15">
@@ -3439,7 +3427,7 @@
         <v>16</v>
       </c>
       <c r="H51" s="17"/>
-      <c r="I51" s="38"/>
+      <c r="I51" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="19.5">
       <c r="A52" s="15">
@@ -3462,7 +3450,7 @@
         <v>16</v>
       </c>
       <c r="H52" s="17"/>
-      <c r="I52" s="38"/>
+      <c r="I52" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="19.5">
       <c r="A53" s="15">
@@ -3485,7 +3473,7 @@
         <v>16</v>
       </c>
       <c r="H53" s="17"/>
-      <c r="I53" s="38"/>
+      <c r="I53" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="19.5">
       <c r="A54" s="15">
@@ -3508,7 +3496,7 @@
         <v>16</v>
       </c>
       <c r="H54" s="17"/>
-      <c r="I54" s="38"/>
+      <c r="I54" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="19.5">
       <c r="A55" s="15">
@@ -3531,7 +3519,7 @@
         <v>16</v>
       </c>
       <c r="H55" s="17"/>
-      <c r="I55" s="38"/>
+      <c r="I55" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="19.5">
       <c r="A56" s="15">
@@ -3554,7 +3542,7 @@
         <v>16</v>
       </c>
       <c r="H56" s="17"/>
-      <c r="I56" s="38"/>
+      <c r="I56" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="19.5">
       <c r="A57" s="15">
@@ -3577,7 +3565,7 @@
         <v>16</v>
       </c>
       <c r="H57" s="17"/>
-      <c r="I57" s="38"/>
+      <c r="I57" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="33.75">
       <c r="A58" s="15">
@@ -3600,7 +3588,7 @@
         <v>16</v>
       </c>
       <c r="H58" s="17"/>
-      <c r="I58" s="38"/>
+      <c r="I58" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="19.5">
       <c r="A59" s="15">
@@ -3623,7 +3611,7 @@
         <v>16</v>
       </c>
       <c r="H59" s="17"/>
-      <c r="I59" s="38"/>
+      <c r="I59" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="19.5">
       <c r="A60" s="15">
@@ -3646,7 +3634,7 @@
         <v>16</v>
       </c>
       <c r="H60" s="17"/>
-      <c r="I60" s="38"/>
+      <c r="I60" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="19.5">
       <c r="A61" s="15">
@@ -3669,7 +3657,7 @@
         <v>16</v>
       </c>
       <c r="H61" s="17"/>
-      <c r="I61" s="38"/>
+      <c r="I61" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="20.25">
       <c r="A62" s="15">
@@ -3692,13 +3680,13 @@
         <v>16</v>
       </c>
       <c r="H62" s="17"/>
-      <c r="I62" s="38"/>
+      <c r="I62" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="19.5" customFormat="1" s="1">
-      <c r="A63" s="44"/>
+      <c r="A63" s="42"/>
       <c r="B63" s="2"/>
-      <c r="C63" s="45"/>
-      <c r="D63" s="46"/>
+      <c r="C63" s="43"/>
+      <c r="D63" s="44"/>
       <c r="E63" s="2"/>
       <c r="F63" s="2"/>
       <c r="G63" s="2"/>
@@ -3743,7 +3731,7 @@
       <c r="H65" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="I65" s="38"/>
+      <c r="I65" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="19.5">
       <c r="A66" s="15">
@@ -3766,7 +3754,7 @@
         <v>16</v>
       </c>
       <c r="H66" s="17"/>
-      <c r="I66" s="38"/>
+      <c r="I66" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="33.75">
       <c r="A67" s="15">
@@ -3789,7 +3777,7 @@
         <v>16</v>
       </c>
       <c r="H67" s="17"/>
-      <c r="I67" s="38"/>
+      <c r="I67" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="33.75">
       <c r="A68" s="15">
@@ -3812,7 +3800,7 @@
         <v>16</v>
       </c>
       <c r="H68" s="17"/>
-      <c r="I68" s="38"/>
+      <c r="I68" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="33.75">
       <c r="A69" s="15">
@@ -3835,7 +3823,7 @@
         <v>16</v>
       </c>
       <c r="H69" s="17"/>
-      <c r="I69" s="38"/>
+      <c r="I69" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="33.75">
       <c r="A70" s="15">
@@ -3858,7 +3846,7 @@
         <v>16</v>
       </c>
       <c r="H70" s="17"/>
-      <c r="I70" s="38"/>
+      <c r="I70" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="33.75">
       <c r="A71" s="15">
@@ -3881,7 +3869,7 @@
         <v>16</v>
       </c>
       <c r="H71" s="17"/>
-      <c r="I71" s="38"/>
+      <c r="I71" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="33.75">
       <c r="A72" s="15">
@@ -3904,7 +3892,7 @@
         <v>16</v>
       </c>
       <c r="H72" s="17"/>
-      <c r="I72" s="38"/>
+      <c r="I72" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="33.75">
       <c r="A73" s="15">
@@ -3927,7 +3915,7 @@
         <v>16</v>
       </c>
       <c r="H73" s="17"/>
-      <c r="I73" s="38"/>
+      <c r="I73" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="33.75">
       <c r="A74" s="15">
@@ -3950,7 +3938,7 @@
         <v>16</v>
       </c>
       <c r="H74" s="17"/>
-      <c r="I74" s="38"/>
+      <c r="I74" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="33.75">
       <c r="A75" s="15">
@@ -3973,7 +3961,7 @@
         <v>16</v>
       </c>
       <c r="H75" s="17"/>
-      <c r="I75" s="38"/>
+      <c r="I75" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="20.25">
       <c r="A76" s="15">
@@ -3996,18 +3984,18 @@
         <v>16</v>
       </c>
       <c r="H76" s="17"/>
-      <c r="I76" s="38"/>
+      <c r="I76" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="19.5">
       <c r="A77" s="21"/>
-      <c r="B77" s="38"/>
+      <c r="B77" s="36"/>
       <c r="C77" s="31"/>
       <c r="D77" s="32"/>
       <c r="E77" s="2"/>
       <c r="F77" s="2"/>
-      <c r="G77" s="38"/>
-      <c r="H77" s="38"/>
-      <c r="I77" s="38"/>
+      <c r="G77" s="36"/>
+      <c r="H77" s="36"/>
+      <c r="I77" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A78" s="11" t="s">
@@ -4047,7 +4035,7 @@
       <c r="H79" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="I79" s="38"/>
+      <c r="I79" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75">
       <c r="A80" s="15">
@@ -4056,8 +4044,8 @@
       <c r="B80" s="16" t="s">
         <v>282</v>
       </c>
-      <c r="C80" s="47">
-        <v>32.1178125</v>
+      <c r="C80" s="45">
+        <v>33.11769675925926</v>
       </c>
       <c r="D80" s="18">
         <v>45374</v>
@@ -4070,7 +4058,7 @@
         <v>16</v>
       </c>
       <c r="H80" s="19"/>
-      <c r="I80" s="38"/>
+      <c r="I80" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18.75">
       <c r="A81" s="15">
@@ -4079,8 +4067,8 @@
       <c r="B81" s="16" t="s">
         <v>282</v>
       </c>
-      <c r="C81" s="47">
-        <v>32.1178125</v>
+      <c r="C81" s="45">
+        <v>33.11769675925926</v>
       </c>
       <c r="D81" s="18">
         <v>45375</v>
@@ -4093,7 +4081,7 @@
         <v>16</v>
       </c>
       <c r="H81" s="19"/>
-      <c r="I81" s="38"/>
+      <c r="I81" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75">
       <c r="A82" s="15">
@@ -4102,8 +4090,8 @@
       <c r="B82" s="16" t="s">
         <v>282</v>
       </c>
-      <c r="C82" s="47">
-        <v>32.1178125</v>
+      <c r="C82" s="45">
+        <v>33.11769675925926</v>
       </c>
       <c r="D82" s="18">
         <v>45376</v>
@@ -4116,7 +4104,7 @@
         <v>16</v>
       </c>
       <c r="H82" s="19"/>
-      <c r="I82" s="38"/>
+      <c r="I82" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75">
       <c r="A83" s="15">
@@ -4125,8 +4113,8 @@
       <c r="B83" s="16" t="s">
         <v>282</v>
       </c>
-      <c r="C83" s="47">
-        <v>32.1178125</v>
+      <c r="C83" s="45">
+        <v>33.11769675925926</v>
       </c>
       <c r="D83" s="18">
         <v>45377</v>
@@ -4139,7 +4127,7 @@
         <v>16</v>
       </c>
       <c r="H83" s="19"/>
-      <c r="I83" s="38"/>
+      <c r="I83" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75">
       <c r="A84" s="15">
@@ -4162,7 +4150,7 @@
         <v>16</v>
       </c>
       <c r="H84" s="17"/>
-      <c r="I84" s="38"/>
+      <c r="I84" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75">
       <c r="A85" s="15">
@@ -4185,7 +4173,7 @@
         <v>16</v>
       </c>
       <c r="H85" s="17"/>
-      <c r="I85" s="38"/>
+      <c r="I85" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75">
       <c r="A86" s="15">
@@ -4208,7 +4196,7 @@
         <v>16</v>
       </c>
       <c r="H86" s="17"/>
-      <c r="I86" s="38"/>
+      <c r="I86" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75">
       <c r="A87" s="15">
@@ -4231,7 +4219,7 @@
         <v>16</v>
       </c>
       <c r="H87" s="17"/>
-      <c r="I87" s="38"/>
+      <c r="I87" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75">
       <c r="A88" s="15">
@@ -4254,7 +4242,7 @@
         <v>16</v>
       </c>
       <c r="H88" s="17"/>
-      <c r="I88" s="38"/>
+      <c r="I88" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75">
       <c r="A89" s="15">
@@ -4277,7 +4265,7 @@
         <v>16</v>
       </c>
       <c r="H89" s="17"/>
-      <c r="I89" s="38"/>
+      <c r="I89" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75">
       <c r="A90" s="15">
@@ -4300,7 +4288,7 @@
         <v>16</v>
       </c>
       <c r="H90" s="17"/>
-      <c r="I90" s="38"/>
+      <c r="I90" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18.75">
       <c r="A91" s="15">
@@ -4323,7 +4311,7 @@
         <v>16</v>
       </c>
       <c r="H91" s="17"/>
-      <c r="I91" s="38"/>
+      <c r="I91" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75">
       <c r="A92" s="15">
@@ -4346,7 +4334,7 @@
         <v>16</v>
       </c>
       <c r="H92" s="17"/>
-      <c r="I92" s="38"/>
+      <c r="I92" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18.75">
       <c r="A93" s="15">
@@ -4369,7 +4357,7 @@
         <v>16</v>
       </c>
       <c r="H93" s="17"/>
-      <c r="I93" s="38"/>
+      <c r="I93" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75">
       <c r="A94" s="15">
@@ -4392,7 +4380,7 @@
         <v>16</v>
       </c>
       <c r="H94" s="17"/>
-      <c r="I94" s="38"/>
+      <c r="I94" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75">
       <c r="A95" s="15">
@@ -4415,7 +4403,7 @@
         <v>16</v>
       </c>
       <c r="H95" s="17"/>
-      <c r="I95" s="38"/>
+      <c r="I95" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75">
       <c r="A96" s="15">
@@ -4438,7 +4426,7 @@
         <v>16</v>
       </c>
       <c r="H96" s="17"/>
-      <c r="I96" s="38"/>
+      <c r="I96" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18.75">
       <c r="A97" s="15">
@@ -4461,7 +4449,7 @@
         <v>16</v>
       </c>
       <c r="H97" s="17"/>
-      <c r="I97" s="38"/>
+      <c r="I97" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18.75">
       <c r="A98" s="15">
@@ -4484,7 +4472,7 @@
         <v>16</v>
       </c>
       <c r="H98" s="17"/>
-      <c r="I98" s="38"/>
+      <c r="I98" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18.75">
       <c r="A99" s="15">
@@ -4507,7 +4495,7 @@
         <v>16</v>
       </c>
       <c r="H99" s="17"/>
-      <c r="I99" s="38"/>
+      <c r="I99" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18.75">
       <c r="A100" s="15">
@@ -4530,7 +4518,7 @@
         <v>16</v>
       </c>
       <c r="H100" s="17"/>
-      <c r="I100" s="38"/>
+      <c r="I100" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18.75">
       <c r="A101" s="15">
@@ -4553,7 +4541,7 @@
         <v>16</v>
       </c>
       <c r="H101" s="17"/>
-      <c r="I101" s="38"/>
+      <c r="I101" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18.75">
       <c r="A102" s="15">
@@ -4576,7 +4564,7 @@
         <v>16</v>
       </c>
       <c r="H102" s="17"/>
-      <c r="I102" s="38"/>
+      <c r="I102" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="33">
       <c r="A103" s="15">
@@ -4599,7 +4587,7 @@
         <v>16</v>
       </c>
       <c r="H103" s="17"/>
-      <c r="I103" s="38"/>
+      <c r="I103" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="33.75">
       <c r="A104" s="15">
@@ -4622,7 +4610,7 @@
         <v>16</v>
       </c>
       <c r="H104" s="17"/>
-      <c r="I104" s="38"/>
+      <c r="I104" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="33">
       <c r="A105" s="15">
@@ -4645,7 +4633,7 @@
         <v>16</v>
       </c>
       <c r="H105" s="17"/>
-      <c r="I105" s="38"/>
+      <c r="I105" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18.75">
       <c r="A106" s="15">
@@ -4668,7 +4656,7 @@
         <v>16</v>
       </c>
       <c r="H106" s="17"/>
-      <c r="I106" s="38"/>
+      <c r="I106" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18.75">
       <c r="A107" s="15">
@@ -4691,7 +4679,7 @@
         <v>16</v>
       </c>
       <c r="H107" s="17"/>
-      <c r="I107" s="38"/>
+      <c r="I107" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="33">
       <c r="A108" s="15">
@@ -4714,7 +4702,7 @@
         <v>16</v>
       </c>
       <c r="H108" s="17"/>
-      <c r="I108" s="38"/>
+      <c r="I108" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18.75">
       <c r="A109" s="15">
@@ -4737,750 +4725,750 @@
         <v>16</v>
       </c>
       <c r="H109" s="17"/>
-      <c r="I109" s="38"/>
+      <c r="I109" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18.75">
       <c r="A110" s="21"/>
-      <c r="B110" s="38"/>
+      <c r="B110" s="36"/>
       <c r="C110" s="31"/>
       <c r="D110" s="32"/>
       <c r="E110" s="2"/>
       <c r="F110" s="2"/>
-      <c r="G110" s="48"/>
-      <c r="H110" s="38"/>
-      <c r="I110" s="38"/>
+      <c r="G110" s="46"/>
+      <c r="H110" s="36"/>
+      <c r="I110" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18.75">
       <c r="A111" s="21"/>
-      <c r="B111" s="38"/>
+      <c r="B111" s="36"/>
       <c r="C111" s="31"/>
       <c r="D111" s="32"/>
       <c r="E111" s="2"/>
       <c r="F111" s="2"/>
-      <c r="G111" s="48"/>
-      <c r="H111" s="38"/>
-      <c r="I111" s="38"/>
+      <c r="G111" s="46"/>
+      <c r="H111" s="36"/>
+      <c r="I111" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18.75">
       <c r="A112" s="21"/>
-      <c r="B112" s="38"/>
+      <c r="B112" s="36"/>
       <c r="C112" s="31"/>
       <c r="D112" s="32"/>
       <c r="E112" s="2"/>
       <c r="F112" s="2"/>
-      <c r="G112" s="48"/>
-      <c r="H112" s="38"/>
-      <c r="I112" s="38"/>
+      <c r="G112" s="46"/>
+      <c r="H112" s="36"/>
+      <c r="I112" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18.75">
       <c r="A113" s="21"/>
-      <c r="B113" s="38"/>
+      <c r="B113" s="36"/>
       <c r="C113" s="31"/>
       <c r="D113" s="32"/>
       <c r="E113" s="2"/>
       <c r="F113" s="2"/>
-      <c r="G113" s="48"/>
-      <c r="H113" s="38"/>
-      <c r="I113" s="38"/>
+      <c r="G113" s="46"/>
+      <c r="H113" s="36"/>
+      <c r="I113" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18.75">
       <c r="A114" s="21"/>
-      <c r="B114" s="38"/>
+      <c r="B114" s="36"/>
       <c r="C114" s="31"/>
       <c r="D114" s="32"/>
       <c r="E114" s="2"/>
       <c r="F114" s="2"/>
-      <c r="G114" s="48"/>
-      <c r="H114" s="38"/>
-      <c r="I114" s="38"/>
+      <c r="G114" s="46"/>
+      <c r="H114" s="36"/>
+      <c r="I114" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18.75">
       <c r="A115" s="21"/>
-      <c r="B115" s="38"/>
+      <c r="B115" s="36"/>
       <c r="C115" s="31"/>
       <c r="D115" s="32"/>
       <c r="E115" s="2"/>
       <c r="F115" s="2"/>
-      <c r="G115" s="48"/>
-      <c r="H115" s="38"/>
-      <c r="I115" s="38"/>
+      <c r="G115" s="46"/>
+      <c r="H115" s="36"/>
+      <c r="I115" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18.75">
       <c r="A116" s="21"/>
-      <c r="B116" s="38"/>
+      <c r="B116" s="36"/>
       <c r="C116" s="31"/>
       <c r="D116" s="32"/>
       <c r="E116" s="2"/>
       <c r="F116" s="2"/>
-      <c r="G116" s="48"/>
-      <c r="H116" s="38"/>
-      <c r="I116" s="38"/>
+      <c r="G116" s="46"/>
+      <c r="H116" s="36"/>
+      <c r="I116" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="18.75">
       <c r="A117" s="21"/>
-      <c r="B117" s="38"/>
+      <c r="B117" s="36"/>
       <c r="C117" s="31"/>
       <c r="D117" s="32"/>
       <c r="E117" s="2"/>
       <c r="F117" s="2"/>
-      <c r="G117" s="48"/>
-      <c r="H117" s="38"/>
-      <c r="I117" s="38"/>
+      <c r="G117" s="46"/>
+      <c r="H117" s="36"/>
+      <c r="I117" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18.75">
       <c r="A118" s="21"/>
-      <c r="B118" s="38"/>
+      <c r="B118" s="36"/>
       <c r="C118" s="31"/>
       <c r="D118" s="32"/>
       <c r="E118" s="2"/>
       <c r="F118" s="2"/>
-      <c r="G118" s="48"/>
-      <c r="H118" s="38"/>
-      <c r="I118" s="38"/>
+      <c r="G118" s="46"/>
+      <c r="H118" s="36"/>
+      <c r="I118" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18.75">
       <c r="A119" s="21"/>
-      <c r="B119" s="38"/>
+      <c r="B119" s="36"/>
       <c r="C119" s="31"/>
       <c r="D119" s="32"/>
       <c r="E119" s="2"/>
       <c r="F119" s="2"/>
-      <c r="G119" s="48"/>
-      <c r="H119" s="38"/>
-      <c r="I119" s="38"/>
+      <c r="G119" s="46"/>
+      <c r="H119" s="36"/>
+      <c r="I119" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18.75">
       <c r="A120" s="21"/>
-      <c r="B120" s="38"/>
+      <c r="B120" s="36"/>
       <c r="C120" s="31"/>
       <c r="D120" s="32"/>
       <c r="E120" s="2"/>
       <c r="F120" s="2"/>
-      <c r="G120" s="48"/>
-      <c r="H120" s="38"/>
-      <c r="I120" s="38"/>
+      <c r="G120" s="46"/>
+      <c r="H120" s="36"/>
+      <c r="I120" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18.75">
       <c r="A121" s="21"/>
-      <c r="B121" s="38"/>
+      <c r="B121" s="36"/>
       <c r="C121" s="31"/>
       <c r="D121" s="32"/>
       <c r="E121" s="2"/>
       <c r="F121" s="2"/>
-      <c r="G121" s="48"/>
-      <c r="H121" s="38"/>
-      <c r="I121" s="38"/>
+      <c r="G121" s="46"/>
+      <c r="H121" s="36"/>
+      <c r="I121" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="18.75">
       <c r="A122" s="21"/>
-      <c r="B122" s="38"/>
+      <c r="B122" s="36"/>
       <c r="C122" s="31"/>
       <c r="D122" s="32"/>
       <c r="E122" s="2"/>
       <c r="F122" s="2"/>
-      <c r="G122" s="48"/>
-      <c r="H122" s="38"/>
-      <c r="I122" s="38"/>
+      <c r="G122" s="46"/>
+      <c r="H122" s="36"/>
+      <c r="I122" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="18.75">
       <c r="A123" s="21"/>
-      <c r="B123" s="38"/>
+      <c r="B123" s="36"/>
       <c r="C123" s="31"/>
       <c r="D123" s="32"/>
       <c r="E123" s="2"/>
       <c r="F123" s="2"/>
-      <c r="G123" s="48"/>
-      <c r="H123" s="38"/>
-      <c r="I123" s="38"/>
+      <c r="G123" s="46"/>
+      <c r="H123" s="36"/>
+      <c r="I123" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="18.75">
       <c r="A124" s="21"/>
-      <c r="B124" s="38"/>
+      <c r="B124" s="36"/>
       <c r="C124" s="31"/>
       <c r="D124" s="32"/>
       <c r="E124" s="2"/>
       <c r="F124" s="2"/>
-      <c r="G124" s="48"/>
-      <c r="H124" s="38"/>
-      <c r="I124" s="38"/>
+      <c r="G124" s="46"/>
+      <c r="H124" s="36"/>
+      <c r="I124" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="18.75">
       <c r="A125" s="21"/>
-      <c r="B125" s="38"/>
+      <c r="B125" s="36"/>
       <c r="C125" s="31"/>
       <c r="D125" s="32"/>
       <c r="E125" s="2"/>
       <c r="F125" s="2"/>
-      <c r="G125" s="48"/>
-      <c r="H125" s="38"/>
-      <c r="I125" s="38"/>
+      <c r="G125" s="46"/>
+      <c r="H125" s="36"/>
+      <c r="I125" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18.75">
       <c r="A126" s="21"/>
-      <c r="B126" s="38"/>
+      <c r="B126" s="36"/>
       <c r="C126" s="31"/>
       <c r="D126" s="32"/>
       <c r="E126" s="2"/>
       <c r="F126" s="2"/>
-      <c r="G126" s="48"/>
-      <c r="H126" s="38"/>
-      <c r="I126" s="38"/>
+      <c r="G126" s="46"/>
+      <c r="H126" s="36"/>
+      <c r="I126" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18.75">
       <c r="A127" s="21"/>
-      <c r="B127" s="38"/>
+      <c r="B127" s="36"/>
       <c r="C127" s="31"/>
       <c r="D127" s="32"/>
       <c r="E127" s="2"/>
       <c r="F127" s="2"/>
-      <c r="G127" s="48"/>
-      <c r="H127" s="38"/>
-      <c r="I127" s="38"/>
+      <c r="G127" s="46"/>
+      <c r="H127" s="36"/>
+      <c r="I127" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18.75">
       <c r="A128" s="21"/>
-      <c r="B128" s="38"/>
+      <c r="B128" s="36"/>
       <c r="C128" s="31"/>
       <c r="D128" s="32"/>
       <c r="E128" s="2"/>
       <c r="F128" s="2"/>
-      <c r="G128" s="48"/>
-      <c r="H128" s="38"/>
-      <c r="I128" s="38"/>
+      <c r="G128" s="46"/>
+      <c r="H128" s="36"/>
+      <c r="I128" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="18.75">
       <c r="A129" s="21"/>
-      <c r="B129" s="38"/>
+      <c r="B129" s="36"/>
       <c r="C129" s="31"/>
       <c r="D129" s="32"/>
       <c r="E129" s="2"/>
       <c r="F129" s="2"/>
-      <c r="G129" s="48"/>
-      <c r="H129" s="38"/>
-      <c r="I129" s="38"/>
+      <c r="G129" s="46"/>
+      <c r="H129" s="36"/>
+      <c r="I129" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="18.75">
       <c r="A130" s="21"/>
-      <c r="B130" s="38"/>
+      <c r="B130" s="36"/>
       <c r="C130" s="31"/>
       <c r="D130" s="32"/>
       <c r="E130" s="2"/>
       <c r="F130" s="2"/>
-      <c r="G130" s="48"/>
-      <c r="H130" s="38"/>
-      <c r="I130" s="38"/>
+      <c r="G130" s="46"/>
+      <c r="H130" s="36"/>
+      <c r="I130" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="131" customHeight="1" ht="18.75">
       <c r="A131" s="21"/>
-      <c r="B131" s="38"/>
+      <c r="B131" s="36"/>
       <c r="C131" s="31"/>
       <c r="D131" s="32"/>
       <c r="E131" s="2"/>
       <c r="F131" s="2"/>
-      <c r="G131" s="48"/>
-      <c r="H131" s="38"/>
-      <c r="I131" s="38"/>
+      <c r="G131" s="46"/>
+      <c r="H131" s="36"/>
+      <c r="I131" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="132" customHeight="1" ht="18.75">
       <c r="A132" s="21"/>
-      <c r="B132" s="38"/>
+      <c r="B132" s="36"/>
       <c r="C132" s="31"/>
       <c r="D132" s="32"/>
       <c r="E132" s="2"/>
       <c r="F132" s="2"/>
-      <c r="G132" s="48"/>
-      <c r="H132" s="38"/>
-      <c r="I132" s="38"/>
+      <c r="G132" s="46"/>
+      <c r="H132" s="36"/>
+      <c r="I132" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="133" customHeight="1" ht="18.75">
       <c r="A133" s="21"/>
-      <c r="B133" s="38"/>
+      <c r="B133" s="36"/>
       <c r="C133" s="31"/>
       <c r="D133" s="32"/>
       <c r="E133" s="2"/>
       <c r="F133" s="2"/>
-      <c r="G133" s="48"/>
-      <c r="H133" s="38"/>
-      <c r="I133" s="38"/>
+      <c r="G133" s="46"/>
+      <c r="H133" s="36"/>
+      <c r="I133" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="18.75">
       <c r="A134" s="21"/>
-      <c r="B134" s="38"/>
+      <c r="B134" s="36"/>
       <c r="C134" s="31"/>
       <c r="D134" s="32"/>
       <c r="E134" s="2"/>
       <c r="F134" s="2"/>
-      <c r="G134" s="48"/>
-      <c r="H134" s="38"/>
-      <c r="I134" s="38"/>
+      <c r="G134" s="46"/>
+      <c r="H134" s="36"/>
+      <c r="I134" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="18.75">
       <c r="A135" s="21"/>
-      <c r="B135" s="38"/>
+      <c r="B135" s="36"/>
       <c r="C135" s="31"/>
       <c r="D135" s="32"/>
       <c r="E135" s="2"/>
       <c r="F135" s="2"/>
-      <c r="G135" s="48"/>
-      <c r="H135" s="38"/>
-      <c r="I135" s="38"/>
+      <c r="G135" s="46"/>
+      <c r="H135" s="36"/>
+      <c r="I135" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="18.75">
       <c r="A136" s="21"/>
-      <c r="B136" s="38"/>
+      <c r="B136" s="36"/>
       <c r="C136" s="31"/>
       <c r="D136" s="32"/>
       <c r="E136" s="2"/>
       <c r="F136" s="2"/>
-      <c r="G136" s="48"/>
-      <c r="H136" s="38"/>
-      <c r="I136" s="38"/>
+      <c r="G136" s="46"/>
+      <c r="H136" s="36"/>
+      <c r="I136" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="18.75">
       <c r="A137" s="21"/>
-      <c r="B137" s="38"/>
+      <c r="B137" s="36"/>
       <c r="C137" s="31"/>
       <c r="D137" s="32"/>
       <c r="E137" s="2"/>
       <c r="F137" s="2"/>
-      <c r="G137" s="48"/>
-      <c r="H137" s="38"/>
-      <c r="I137" s="38"/>
+      <c r="G137" s="46"/>
+      <c r="H137" s="36"/>
+      <c r="I137" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="18.75">
       <c r="A138" s="21"/>
-      <c r="B138" s="38"/>
+      <c r="B138" s="36"/>
       <c r="C138" s="31"/>
       <c r="D138" s="32"/>
       <c r="E138" s="2"/>
       <c r="F138" s="2"/>
-      <c r="G138" s="48"/>
-      <c r="H138" s="38"/>
-      <c r="I138" s="38"/>
+      <c r="G138" s="46"/>
+      <c r="H138" s="36"/>
+      <c r="I138" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="18.75">
       <c r="A139" s="21"/>
-      <c r="B139" s="38"/>
+      <c r="B139" s="36"/>
       <c r="C139" s="31"/>
       <c r="D139" s="32"/>
       <c r="E139" s="2"/>
       <c r="F139" s="2"/>
-      <c r="G139" s="48"/>
-      <c r="H139" s="38"/>
-      <c r="I139" s="38"/>
+      <c r="G139" s="46"/>
+      <c r="H139" s="36"/>
+      <c r="I139" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="18.75">
       <c r="A140" s="21"/>
-      <c r="B140" s="38"/>
+      <c r="B140" s="36"/>
       <c r="C140" s="31"/>
       <c r="D140" s="32"/>
       <c r="E140" s="2"/>
       <c r="F140" s="2"/>
-      <c r="G140" s="48"/>
-      <c r="H140" s="38"/>
-      <c r="I140" s="38"/>
+      <c r="G140" s="46"/>
+      <c r="H140" s="36"/>
+      <c r="I140" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="18.75">
       <c r="A141" s="21"/>
-      <c r="B141" s="38"/>
+      <c r="B141" s="36"/>
       <c r="C141" s="31"/>
       <c r="D141" s="32"/>
       <c r="E141" s="2"/>
       <c r="F141" s="2"/>
-      <c r="G141" s="48"/>
-      <c r="H141" s="38"/>
-      <c r="I141" s="38"/>
+      <c r="G141" s="46"/>
+      <c r="H141" s="36"/>
+      <c r="I141" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="18.75">
       <c r="A142" s="21"/>
-      <c r="B142" s="38"/>
+      <c r="B142" s="36"/>
       <c r="C142" s="31"/>
       <c r="D142" s="32"/>
       <c r="E142" s="2"/>
       <c r="F142" s="2"/>
-      <c r="G142" s="48"/>
-      <c r="H142" s="38"/>
-      <c r="I142" s="38"/>
+      <c r="G142" s="46"/>
+      <c r="H142" s="36"/>
+      <c r="I142" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="18.75">
       <c r="A143" s="21"/>
-      <c r="B143" s="38"/>
+      <c r="B143" s="36"/>
       <c r="C143" s="31"/>
       <c r="D143" s="32"/>
       <c r="E143" s="2"/>
       <c r="F143" s="2"/>
-      <c r="G143" s="48"/>
-      <c r="H143" s="38"/>
-      <c r="I143" s="38"/>
+      <c r="G143" s="46"/>
+      <c r="H143" s="36"/>
+      <c r="I143" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="144" customHeight="1" ht="18.75">
       <c r="A144" s="21"/>
-      <c r="B144" s="38"/>
+      <c r="B144" s="36"/>
       <c r="C144" s="31"/>
       <c r="D144" s="32"/>
       <c r="E144" s="2"/>
       <c r="F144" s="2"/>
-      <c r="G144" s="48"/>
-      <c r="H144" s="38"/>
-      <c r="I144" s="38"/>
+      <c r="G144" s="46"/>
+      <c r="H144" s="36"/>
+      <c r="I144" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="145" customHeight="1" ht="18.75">
       <c r="A145" s="21"/>
-      <c r="B145" s="38"/>
+      <c r="B145" s="36"/>
       <c r="C145" s="31"/>
       <c r="D145" s="32"/>
       <c r="E145" s="2"/>
       <c r="F145" s="2"/>
-      <c r="G145" s="48"/>
-      <c r="H145" s="38"/>
-      <c r="I145" s="38"/>
+      <c r="G145" s="46"/>
+      <c r="H145" s="36"/>
+      <c r="I145" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="146" customHeight="1" ht="18.75">
       <c r="A146" s="21"/>
-      <c r="B146" s="38"/>
+      <c r="B146" s="36"/>
       <c r="C146" s="31"/>
       <c r="D146" s="32"/>
       <c r="E146" s="2"/>
       <c r="F146" s="2"/>
-      <c r="G146" s="48"/>
-      <c r="H146" s="38"/>
-      <c r="I146" s="38"/>
+      <c r="G146" s="46"/>
+      <c r="H146" s="36"/>
+      <c r="I146" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="147" customHeight="1" ht="18.75">
       <c r="A147" s="21"/>
-      <c r="B147" s="38"/>
+      <c r="B147" s="36"/>
       <c r="C147" s="31"/>
       <c r="D147" s="32"/>
       <c r="E147" s="2"/>
       <c r="F147" s="2"/>
-      <c r="G147" s="48"/>
-      <c r="H147" s="38"/>
-      <c r="I147" s="38"/>
+      <c r="G147" s="46"/>
+      <c r="H147" s="36"/>
+      <c r="I147" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="148" customHeight="1" ht="18.75">
       <c r="A148" s="21"/>
-      <c r="B148" s="38"/>
+      <c r="B148" s="36"/>
       <c r="C148" s="31"/>
       <c r="D148" s="32"/>
       <c r="E148" s="2"/>
       <c r="F148" s="2"/>
-      <c r="G148" s="48"/>
-      <c r="H148" s="38"/>
-      <c r="I148" s="38"/>
+      <c r="G148" s="46"/>
+      <c r="H148" s="36"/>
+      <c r="I148" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="149" customHeight="1" ht="18.75">
       <c r="A149" s="21"/>
-      <c r="B149" s="38"/>
+      <c r="B149" s="36"/>
       <c r="C149" s="31"/>
       <c r="D149" s="32"/>
       <c r="E149" s="2"/>
       <c r="F149" s="2"/>
-      <c r="G149" s="48"/>
-      <c r="H149" s="38"/>
-      <c r="I149" s="38"/>
+      <c r="G149" s="46"/>
+      <c r="H149" s="36"/>
+      <c r="I149" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="150" customHeight="1" ht="18.75">
       <c r="A150" s="21"/>
-      <c r="B150" s="38"/>
+      <c r="B150" s="36"/>
       <c r="C150" s="31"/>
       <c r="D150" s="32"/>
       <c r="E150" s="2"/>
       <c r="F150" s="2"/>
-      <c r="G150" s="48"/>
-      <c r="H150" s="38"/>
-      <c r="I150" s="38"/>
+      <c r="G150" s="46"/>
+      <c r="H150" s="36"/>
+      <c r="I150" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="151" customHeight="1" ht="18.75">
       <c r="A151" s="21"/>
-      <c r="B151" s="38"/>
+      <c r="B151" s="36"/>
       <c r="C151" s="31"/>
       <c r="D151" s="32"/>
       <c r="E151" s="2"/>
       <c r="F151" s="2"/>
-      <c r="G151" s="48"/>
-      <c r="H151" s="38"/>
-      <c r="I151" s="38"/>
+      <c r="G151" s="46"/>
+      <c r="H151" s="36"/>
+      <c r="I151" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="152" customHeight="1" ht="18.75">
       <c r="A152" s="21"/>
-      <c r="B152" s="38"/>
+      <c r="B152" s="36"/>
       <c r="C152" s="31"/>
       <c r="D152" s="32"/>
       <c r="E152" s="2"/>
       <c r="F152" s="2"/>
-      <c r="G152" s="48"/>
-      <c r="H152" s="38"/>
-      <c r="I152" s="38"/>
+      <c r="G152" s="46"/>
+      <c r="H152" s="36"/>
+      <c r="I152" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="153" customHeight="1" ht="18.75">
       <c r="A153" s="21"/>
-      <c r="B153" s="38"/>
+      <c r="B153" s="36"/>
       <c r="C153" s="31"/>
       <c r="D153" s="32"/>
       <c r="E153" s="2"/>
       <c r="F153" s="2"/>
-      <c r="G153" s="48"/>
-      <c r="H153" s="38"/>
-      <c r="I153" s="38"/>
+      <c r="G153" s="46"/>
+      <c r="H153" s="36"/>
+      <c r="I153" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="154" customHeight="1" ht="18.75">
       <c r="A154" s="21"/>
-      <c r="B154" s="38"/>
+      <c r="B154" s="36"/>
       <c r="C154" s="31"/>
       <c r="D154" s="32"/>
       <c r="E154" s="2"/>
       <c r="F154" s="2"/>
-      <c r="G154" s="48"/>
-      <c r="H154" s="38"/>
-      <c r="I154" s="38"/>
+      <c r="G154" s="46"/>
+      <c r="H154" s="36"/>
+      <c r="I154" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="18.75">
       <c r="A155" s="21"/>
-      <c r="B155" s="38"/>
+      <c r="B155" s="36"/>
       <c r="C155" s="31"/>
       <c r="D155" s="32"/>
       <c r="E155" s="2"/>
       <c r="F155" s="2"/>
-      <c r="G155" s="48"/>
-      <c r="H155" s="38"/>
-      <c r="I155" s="38"/>
+      <c r="G155" s="46"/>
+      <c r="H155" s="36"/>
+      <c r="I155" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="156" customHeight="1" ht="18.75">
       <c r="A156" s="21"/>
-      <c r="B156" s="38"/>
+      <c r="B156" s="36"/>
       <c r="C156" s="31"/>
       <c r="D156" s="32"/>
       <c r="E156" s="2"/>
       <c r="F156" s="2"/>
-      <c r="G156" s="48"/>
-      <c r="H156" s="38"/>
-      <c r="I156" s="38"/>
+      <c r="G156" s="46"/>
+      <c r="H156" s="36"/>
+      <c r="I156" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="157" customHeight="1" ht="18.75">
       <c r="A157" s="21"/>
-      <c r="B157" s="38"/>
+      <c r="B157" s="36"/>
       <c r="C157" s="31"/>
       <c r="D157" s="32"/>
       <c r="E157" s="2"/>
       <c r="F157" s="2"/>
-      <c r="G157" s="48"/>
-      <c r="H157" s="38"/>
-      <c r="I157" s="38"/>
+      <c r="G157" s="46"/>
+      <c r="H157" s="36"/>
+      <c r="I157" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="158" customHeight="1" ht="18.75">
       <c r="A158" s="21"/>
-      <c r="B158" s="38"/>
+      <c r="B158" s="36"/>
       <c r="C158" s="31"/>
       <c r="D158" s="32"/>
       <c r="E158" s="2"/>
       <c r="F158" s="2"/>
-      <c r="G158" s="48"/>
-      <c r="H158" s="38"/>
-      <c r="I158" s="38"/>
+      <c r="G158" s="46"/>
+      <c r="H158" s="36"/>
+      <c r="I158" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="159" customHeight="1" ht="18.75">
       <c r="A159" s="21"/>
-      <c r="B159" s="38"/>
+      <c r="B159" s="36"/>
       <c r="C159" s="31"/>
       <c r="D159" s="32"/>
       <c r="E159" s="2"/>
       <c r="F159" s="2"/>
-      <c r="G159" s="48"/>
-      <c r="H159" s="38"/>
-      <c r="I159" s="38"/>
+      <c r="G159" s="46"/>
+      <c r="H159" s="36"/>
+      <c r="I159" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="160" customHeight="1" ht="18.75">
       <c r="A160" s="21"/>
-      <c r="B160" s="38"/>
+      <c r="B160" s="36"/>
       <c r="C160" s="31"/>
       <c r="D160" s="32"/>
       <c r="E160" s="2"/>
       <c r="F160" s="2"/>
-      <c r="G160" s="48"/>
-      <c r="H160" s="38"/>
-      <c r="I160" s="38"/>
+      <c r="G160" s="46"/>
+      <c r="H160" s="36"/>
+      <c r="I160" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="18.75">
       <c r="A161" s="21"/>
-      <c r="B161" s="38"/>
+      <c r="B161" s="36"/>
       <c r="C161" s="31"/>
       <c r="D161" s="32"/>
       <c r="E161" s="2"/>
       <c r="F161" s="2"/>
-      <c r="G161" s="48"/>
-      <c r="H161" s="38"/>
-      <c r="I161" s="38"/>
+      <c r="G161" s="46"/>
+      <c r="H161" s="36"/>
+      <c r="I161" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="18.75">
       <c r="A162" s="21"/>
-      <c r="B162" s="38"/>
+      <c r="B162" s="36"/>
       <c r="C162" s="31"/>
       <c r="D162" s="32"/>
       <c r="E162" s="2"/>
       <c r="F162" s="2"/>
-      <c r="G162" s="48"/>
-      <c r="H162" s="38"/>
-      <c r="I162" s="38"/>
+      <c r="G162" s="46"/>
+      <c r="H162" s="36"/>
+      <c r="I162" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="18.75">
       <c r="A163" s="21"/>
-      <c r="B163" s="38"/>
+      <c r="B163" s="36"/>
       <c r="C163" s="31"/>
       <c r="D163" s="32"/>
       <c r="E163" s="2"/>
       <c r="F163" s="2"/>
-      <c r="G163" s="48"/>
-      <c r="H163" s="38"/>
-      <c r="I163" s="38"/>
+      <c r="G163" s="46"/>
+      <c r="H163" s="36"/>
+      <c r="I163" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="18.75">
       <c r="A164" s="21"/>
-      <c r="B164" s="38"/>
+      <c r="B164" s="36"/>
       <c r="C164" s="31"/>
       <c r="D164" s="32"/>
       <c r="E164" s="2"/>
       <c r="F164" s="2"/>
-      <c r="G164" s="48"/>
-      <c r="H164" s="38"/>
-      <c r="I164" s="38"/>
+      <c r="G164" s="46"/>
+      <c r="H164" s="36"/>
+      <c r="I164" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="18.75">
       <c r="A165" s="21"/>
-      <c r="B165" s="38"/>
+      <c r="B165" s="36"/>
       <c r="C165" s="31"/>
       <c r="D165" s="32"/>
       <c r="E165" s="2"/>
       <c r="F165" s="2"/>
-      <c r="G165" s="48"/>
-      <c r="H165" s="38"/>
-      <c r="I165" s="38"/>
+      <c r="G165" s="46"/>
+      <c r="H165" s="36"/>
+      <c r="I165" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="18.75">
       <c r="A166" s="21"/>
-      <c r="B166" s="38"/>
+      <c r="B166" s="36"/>
       <c r="C166" s="31"/>
       <c r="D166" s="32"/>
       <c r="E166" s="2"/>
       <c r="F166" s="2"/>
-      <c r="G166" s="48"/>
-      <c r="H166" s="38"/>
-      <c r="I166" s="38"/>
+      <c r="G166" s="46"/>
+      <c r="H166" s="36"/>
+      <c r="I166" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="18.75">
       <c r="A167" s="21"/>
-      <c r="B167" s="38"/>
+      <c r="B167" s="36"/>
       <c r="C167" s="31"/>
       <c r="D167" s="32"/>
       <c r="E167" s="2"/>
       <c r="F167" s="2"/>
-      <c r="G167" s="48"/>
-      <c r="H167" s="38"/>
-      <c r="I167" s="38"/>
+      <c r="G167" s="46"/>
+      <c r="H167" s="36"/>
+      <c r="I167" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="18.75">
       <c r="A168" s="21"/>
-      <c r="B168" s="38"/>
+      <c r="B168" s="36"/>
       <c r="C168" s="31"/>
       <c r="D168" s="32"/>
       <c r="E168" s="2"/>
       <c r="F168" s="2"/>
-      <c r="G168" s="48"/>
-      <c r="H168" s="38"/>
-      <c r="I168" s="38"/>
+      <c r="G168" s="46"/>
+      <c r="H168" s="36"/>
+      <c r="I168" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="18.75">
       <c r="A169" s="21"/>
-      <c r="B169" s="38"/>
+      <c r="B169" s="36"/>
       <c r="C169" s="31"/>
       <c r="D169" s="32"/>
       <c r="E169" s="2"/>
       <c r="F169" s="2"/>
-      <c r="G169" s="48"/>
-      <c r="H169" s="38"/>
-      <c r="I169" s="38"/>
+      <c r="G169" s="46"/>
+      <c r="H169" s="36"/>
+      <c r="I169" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="18.75">
       <c r="A170" s="21"/>
-      <c r="B170" s="38"/>
+      <c r="B170" s="36"/>
       <c r="C170" s="31"/>
       <c r="D170" s="32"/>
       <c r="E170" s="2"/>
       <c r="F170" s="2"/>
-      <c r="G170" s="48"/>
-      <c r="H170" s="38"/>
-      <c r="I170" s="38"/>
+      <c r="G170" s="46"/>
+      <c r="H170" s="36"/>
+      <c r="I170" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="18.75">
       <c r="A171" s="21"/>
-      <c r="B171" s="38"/>
+      <c r="B171" s="36"/>
       <c r="C171" s="31"/>
       <c r="D171" s="32"/>
       <c r="E171" s="2"/>
       <c r="F171" s="2"/>
-      <c r="G171" s="48"/>
-      <c r="H171" s="38"/>
-      <c r="I171" s="38"/>
+      <c r="G171" s="46"/>
+      <c r="H171" s="36"/>
+      <c r="I171" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="18.75">
       <c r="A172" s="21"/>
-      <c r="B172" s="38"/>
+      <c r="B172" s="36"/>
       <c r="C172" s="31"/>
       <c r="D172" s="32"/>
       <c r="E172" s="2"/>
       <c r="F172" s="2"/>
-      <c r="G172" s="48"/>
-      <c r="H172" s="38"/>
-      <c r="I172" s="38"/>
+      <c r="G172" s="46"/>
+      <c r="H172" s="36"/>
+      <c r="I172" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="18.75">
       <c r="A173" s="21"/>
-      <c r="B173" s="38"/>
+      <c r="B173" s="36"/>
       <c r="C173" s="31"/>
       <c r="D173" s="32"/>
       <c r="E173" s="2"/>
       <c r="F173" s="2"/>
-      <c r="G173" s="48"/>
-      <c r="H173" s="38"/>
-      <c r="I173" s="38"/>
+      <c r="G173" s="46"/>
+      <c r="H173" s="36"/>
+      <c r="I173" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="18.75">
       <c r="A174" s="21"/>
-      <c r="B174" s="38"/>
+      <c r="B174" s="36"/>
       <c r="C174" s="31"/>
       <c r="D174" s="32"/>
       <c r="E174" s="2"/>
       <c r="F174" s="2"/>
-      <c r="G174" s="48"/>
-      <c r="H174" s="38"/>
-      <c r="I174" s="38"/>
+      <c r="G174" s="46"/>
+      <c r="H174" s="36"/>
+      <c r="I174" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="18.75">
       <c r="A175" s="21"/>
-      <c r="B175" s="38"/>
+      <c r="B175" s="36"/>
       <c r="C175" s="31"/>
       <c r="D175" s="32"/>
       <c r="E175" s="2"/>
       <c r="F175" s="2"/>
-      <c r="G175" s="48"/>
-      <c r="H175" s="38"/>
-      <c r="I175" s="38"/>
+      <c r="G175" s="46"/>
+      <c r="H175" s="36"/>
+      <c r="I175" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="18.75">
       <c r="A176" s="21"/>
       <c r="B176" s="2"/>
-      <c r="C176" s="49"/>
+      <c r="C176" s="47"/>
       <c r="D176" s="32"/>
       <c r="E176" s="2"/>
       <c r="F176" s="2"/>
-      <c r="G176" s="38"/>
-      <c r="H176" s="38"/>
-      <c r="I176" s="38"/>
+      <c r="G176" s="36"/>
+      <c r="H176" s="36"/>
+      <c r="I176" s="36"/>
     </row>
     <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A177" s="44"/>
+      <c r="A177" s="42"/>
       <c r="B177" s="2"/>
-      <c r="C177" s="45"/>
-      <c r="D177" s="46"/>
+      <c r="C177" s="43"/>
+      <c r="D177" s="44"/>
       <c r="E177" s="2"/>
       <c r="F177" s="2"/>
       <c r="G177" s="2"/>
@@ -5488,10 +5476,10 @@
       <c r="I177" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A178" s="44"/>
+      <c r="A178" s="42"/>
       <c r="B178" s="2"/>
-      <c r="C178" s="45"/>
-      <c r="D178" s="46"/>
+      <c r="C178" s="43"/>
+      <c r="D178" s="44"/>
       <c r="E178" s="2"/>
       <c r="F178" s="2"/>
       <c r="G178" s="2"/>
@@ -5499,10 +5487,10 @@
       <c r="I178" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A179" s="44"/>
+      <c r="A179" s="42"/>
       <c r="B179" s="2"/>
-      <c r="C179" s="45"/>
-      <c r="D179" s="46"/>
+      <c r="C179" s="43"/>
+      <c r="D179" s="44"/>
       <c r="E179" s="2"/>
       <c r="F179" s="2"/>
       <c r="G179" s="2"/>
@@ -5510,10 +5498,10 @@
       <c r="I179" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A180" s="44"/>
+      <c r="A180" s="42"/>
       <c r="B180" s="2"/>
-      <c r="C180" s="45"/>
-      <c r="D180" s="46"/>
+      <c r="C180" s="43"/>
+      <c r="D180" s="44"/>
       <c r="E180" s="2"/>
       <c r="F180" s="2"/>
       <c r="G180" s="2"/>
@@ -5521,10 +5509,10 @@
       <c r="I180" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A181" s="44"/>
+      <c r="A181" s="42"/>
       <c r="B181" s="2"/>
-      <c r="C181" s="45"/>
-      <c r="D181" s="46"/>
+      <c r="C181" s="43"/>
+      <c r="D181" s="44"/>
       <c r="E181" s="2"/>
       <c r="F181" s="2"/>
       <c r="G181" s="2"/>
@@ -5532,10 +5520,10 @@
       <c r="I181" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A182" s="44"/>
+      <c r="A182" s="42"/>
       <c r="B182" s="2"/>
-      <c r="C182" s="45"/>
-      <c r="D182" s="46"/>
+      <c r="C182" s="43"/>
+      <c r="D182" s="44"/>
       <c r="E182" s="2"/>
       <c r="F182" s="2"/>
       <c r="G182" s="2"/>
@@ -5543,10 +5531,10 @@
       <c r="I182" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A183" s="44"/>
+      <c r="A183" s="42"/>
       <c r="B183" s="2"/>
-      <c r="C183" s="45"/>
-      <c r="D183" s="46"/>
+      <c r="C183" s="43"/>
+      <c r="D183" s="44"/>
       <c r="E183" s="2"/>
       <c r="F183" s="2"/>
       <c r="G183" s="2"/>
@@ -5554,10 +5542,10 @@
       <c r="I183" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A184" s="44"/>
+      <c r="A184" s="42"/>
       <c r="B184" s="2"/>
-      <c r="C184" s="45"/>
-      <c r="D184" s="46"/>
+      <c r="C184" s="43"/>
+      <c r="D184" s="44"/>
       <c r="E184" s="2"/>
       <c r="F184" s="2"/>
       <c r="G184" s="2"/>
@@ -5565,10 +5553,10 @@
       <c r="I184" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A185" s="44"/>
+      <c r="A185" s="42"/>
       <c r="B185" s="2"/>
-      <c r="C185" s="45"/>
-      <c r="D185" s="46"/>
+      <c r="C185" s="43"/>
+      <c r="D185" s="44"/>
       <c r="E185" s="2"/>
       <c r="F185" s="2"/>
       <c r="G185" s="2"/>
@@ -5576,10 +5564,10 @@
       <c r="I185" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A186" s="44"/>
+      <c r="A186" s="42"/>
       <c r="B186" s="2"/>
-      <c r="C186" s="45"/>
-      <c r="D186" s="46"/>
+      <c r="C186" s="43"/>
+      <c r="D186" s="44"/>
       <c r="E186" s="2"/>
       <c r="F186" s="2"/>
       <c r="G186" s="2"/>
@@ -5587,10 +5575,10 @@
       <c r="I186" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A187" s="44"/>
+      <c r="A187" s="42"/>
       <c r="B187" s="2"/>
-      <c r="C187" s="45"/>
-      <c r="D187" s="46"/>
+      <c r="C187" s="43"/>
+      <c r="D187" s="44"/>
       <c r="E187" s="2"/>
       <c r="F187" s="2"/>
       <c r="G187" s="2"/>
@@ -5598,10 +5586,10 @@
       <c r="I187" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A188" s="44"/>
+      <c r="A188" s="42"/>
       <c r="B188" s="2"/>
-      <c r="C188" s="45"/>
-      <c r="D188" s="46"/>
+      <c r="C188" s="43"/>
+      <c r="D188" s="44"/>
       <c r="E188" s="2"/>
       <c r="F188" s="2"/>
       <c r="G188" s="2"/>
@@ -5609,10 +5597,10 @@
       <c r="I188" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A189" s="44"/>
+      <c r="A189" s="42"/>
       <c r="B189" s="2"/>
-      <c r="C189" s="45"/>
-      <c r="D189" s="46"/>
+      <c r="C189" s="43"/>
+      <c r="D189" s="44"/>
       <c r="E189" s="2"/>
       <c r="F189" s="2"/>
       <c r="G189" s="2"/>
@@ -5620,10 +5608,10 @@
       <c r="I189" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A190" s="44"/>
+      <c r="A190" s="42"/>
       <c r="B190" s="2"/>
-      <c r="C190" s="45"/>
-      <c r="D190" s="46"/>
+      <c r="C190" s="43"/>
+      <c r="D190" s="44"/>
       <c r="E190" s="2"/>
       <c r="F190" s="2"/>
       <c r="G190" s="2"/>
@@ -5631,10 +5619,10 @@
       <c r="I190" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A191" s="44"/>
+      <c r="A191" s="42"/>
       <c r="B191" s="2"/>
-      <c r="C191" s="45"/>
-      <c r="D191" s="46"/>
+      <c r="C191" s="43"/>
+      <c r="D191" s="44"/>
       <c r="E191" s="2"/>
       <c r="F191" s="2"/>
       <c r="G191" s="2"/>
@@ -5642,10 +5630,10 @@
       <c r="I191" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A192" s="44"/>
+      <c r="A192" s="42"/>
       <c r="B192" s="2"/>
-      <c r="C192" s="45"/>
-      <c r="D192" s="46"/>
+      <c r="C192" s="43"/>
+      <c r="D192" s="44"/>
       <c r="E192" s="2"/>
       <c r="F192" s="2"/>
       <c r="G192" s="2"/>
@@ -5653,10 +5641,10 @@
       <c r="I192" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A193" s="44"/>
+      <c r="A193" s="42"/>
       <c r="B193" s="2"/>
-      <c r="C193" s="45"/>
-      <c r="D193" s="46"/>
+      <c r="C193" s="43"/>
+      <c r="D193" s="44"/>
       <c r="E193" s="2"/>
       <c r="F193" s="2"/>
       <c r="G193" s="2"/>
@@ -5664,10 +5652,10 @@
       <c r="I193" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A194" s="44"/>
+      <c r="A194" s="42"/>
       <c r="B194" s="2"/>
-      <c r="C194" s="45"/>
-      <c r="D194" s="46"/>
+      <c r="C194" s="43"/>
+      <c r="D194" s="44"/>
       <c r="E194" s="2"/>
       <c r="F194" s="2"/>
       <c r="G194" s="2"/>
@@ -5675,10 +5663,10 @@
       <c r="I194" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A195" s="44"/>
+      <c r="A195" s="42"/>
       <c r="B195" s="2"/>
-      <c r="C195" s="45"/>
-      <c r="D195" s="46"/>
+      <c r="C195" s="43"/>
+      <c r="D195" s="44"/>
       <c r="E195" s="2"/>
       <c r="F195" s="2"/>
       <c r="G195" s="2"/>
@@ -5686,10 +5674,10 @@
       <c r="I195" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A196" s="44"/>
+      <c r="A196" s="42"/>
       <c r="B196" s="2"/>
-      <c r="C196" s="45"/>
-      <c r="D196" s="46"/>
+      <c r="C196" s="43"/>
+      <c r="D196" s="44"/>
       <c r="E196" s="2"/>
       <c r="F196" s="2"/>
       <c r="G196" s="2"/>
@@ -5697,10 +5685,10 @@
       <c r="I196" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A197" s="44"/>
+      <c r="A197" s="42"/>
       <c r="B197" s="2"/>
-      <c r="C197" s="45"/>
-      <c r="D197" s="46"/>
+      <c r="C197" s="43"/>
+      <c r="D197" s="44"/>
       <c r="E197" s="2"/>
       <c r="F197" s="2"/>
       <c r="G197" s="2"/>
@@ -5708,10 +5696,10 @@
       <c r="I197" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A198" s="44"/>
+      <c r="A198" s="42"/>
       <c r="B198" s="2"/>
-      <c r="C198" s="45"/>
-      <c r="D198" s="46"/>
+      <c r="C198" s="43"/>
+      <c r="D198" s="44"/>
       <c r="E198" s="2"/>
       <c r="F198" s="2"/>
       <c r="G198" s="2"/>
@@ -5719,10 +5707,10 @@
       <c r="I198" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A199" s="44"/>
+      <c r="A199" s="42"/>
       <c r="B199" s="2"/>
-      <c r="C199" s="45"/>
-      <c r="D199" s="46"/>
+      <c r="C199" s="43"/>
+      <c r="D199" s="44"/>
       <c r="E199" s="2"/>
       <c r="F199" s="2"/>
       <c r="G199" s="2"/>
@@ -5730,10 +5718,10 @@
       <c r="I199" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="200" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A200" s="44"/>
+      <c r="A200" s="42"/>
       <c r="B200" s="2"/>
-      <c r="C200" s="45"/>
-      <c r="D200" s="46"/>
+      <c r="C200" s="43"/>
+      <c r="D200" s="44"/>
       <c r="E200" s="2"/>
       <c r="F200" s="2"/>
       <c r="G200" s="2"/>
@@ -5741,10 +5729,10 @@
       <c r="I200" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="201" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A201" s="44"/>
+      <c r="A201" s="42"/>
       <c r="B201" s="2"/>
-      <c r="C201" s="45"/>
-      <c r="D201" s="46"/>
+      <c r="C201" s="43"/>
+      <c r="D201" s="44"/>
       <c r="E201" s="2"/>
       <c r="F201" s="2"/>
       <c r="G201" s="2"/>
@@ -5752,10 +5740,10 @@
       <c r="I201" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="202" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A202" s="44"/>
+      <c r="A202" s="42"/>
       <c r="B202" s="2"/>
-      <c r="C202" s="45"/>
-      <c r="D202" s="46"/>
+      <c r="C202" s="43"/>
+      <c r="D202" s="44"/>
       <c r="E202" s="2"/>
       <c r="F202" s="2"/>
       <c r="G202" s="2"/>
@@ -5763,10 +5751,10 @@
       <c r="I202" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="203" customHeight="1" ht="18.75" customFormat="1" s="1">
-      <c r="A203" s="44"/>
+      <c r="A203" s="42"/>
       <c r="B203" s="2"/>
-      <c r="C203" s="45"/>
-      <c r="D203" s="46"/>
+      <c r="C203" s="43"/>
+      <c r="D203" s="44"/>
       <c r="E203" s="2"/>
       <c r="F203" s="2"/>
       <c r="G203" s="2"/>
@@ -5794,11 +5782,11 @@
   <cols>
     <col min="1" max="1" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="24" width="43.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="35" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="36" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="34" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="35" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="6" max="6" style="24" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="37" width="16.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="23" width="16.433571428571426" customWidth="1" bestFit="1"/>
     <col min="8" max="8" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
@@ -6274,7 +6262,9 @@
       <c r="E22" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F22" s="17"/>
+      <c r="F22" s="17" t="s">
+        <v>16</v>
+      </c>
       <c r="G22" s="20"/>
       <c r="H22" s="2"/>
     </row>
@@ -6294,7 +6284,9 @@
       <c r="E23" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F23" s="17"/>
+      <c r="F23" s="17" t="s">
+        <v>16</v>
+      </c>
       <c r="G23" s="20"/>
       <c r="H23" s="2"/>
     </row>
@@ -6314,7 +6306,9 @@
       <c r="E24" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F24" s="17"/>
+      <c r="F24" s="17" t="s">
+        <v>16</v>
+      </c>
       <c r="G24" s="20"/>
       <c r="H24" s="2"/>
     </row>
@@ -6334,7 +6328,9 @@
       <c r="E25" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F25" s="17"/>
+      <c r="F25" s="17" t="s">
+        <v>16</v>
+      </c>
       <c r="G25" s="20">
         <v>1</v>
       </c>
@@ -6356,7 +6352,9 @@
       <c r="E26" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="F26" s="17"/>
+      <c r="F26" s="17" t="s">
+        <v>16</v>
+      </c>
       <c r="G26" s="20">
         <v>2</v>
       </c>
@@ -7217,7 +7215,7 @@
       <c r="D69" s="32"/>
       <c r="E69" s="2"/>
       <c r="F69" s="22"/>
-      <c r="G69" s="33"/>
+      <c r="G69" s="21"/>
       <c r="H69" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="29" customFormat="1" s="1">
@@ -8797,7 +8795,7 @@
       <c r="B148" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="C148" s="34" t="s">
+      <c r="C148" s="33" t="s">
         <v>179</v>
       </c>
       <c r="D148" s="18">
@@ -8817,7 +8815,7 @@
       <c r="B149" s="17" t="s">
         <v>181</v>
       </c>
-      <c r="C149" s="34" t="s">
+      <c r="C149" s="33" t="s">
         <v>179</v>
       </c>
       <c r="D149" s="18">
@@ -8837,7 +8835,7 @@
       <c r="B150" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="C150" s="34" t="s">
+      <c r="C150" s="33" t="s">
         <v>179</v>
       </c>
       <c r="D150" s="18">
@@ -8857,7 +8855,7 @@
       <c r="B151" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="C151" s="34" t="s">
+      <c r="C151" s="33" t="s">
         <v>179</v>
       </c>
       <c r="D151" s="18">
@@ -8877,7 +8875,7 @@
       <c r="B152" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="C152" s="34" t="s">
+      <c r="C152" s="33" t="s">
         <v>179</v>
       </c>
       <c r="D152" s="18">
@@ -8897,7 +8895,7 @@
       <c r="B153" s="17" t="s">
         <v>189</v>
       </c>
-      <c r="C153" s="34" t="s">
+      <c r="C153" s="33" t="s">
         <v>179</v>
       </c>
       <c r="D153" s="18">
@@ -8917,7 +8915,7 @@
       <c r="D154" s="32"/>
       <c r="E154" s="2"/>
       <c r="F154" s="22"/>
-      <c r="G154" s="33"/>
+      <c r="G154" s="21"/>
       <c r="H154" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="18.75">
@@ -8927,7 +8925,7 @@
       <c r="D155" s="32"/>
       <c r="E155" s="2"/>
       <c r="F155" s="22"/>
-      <c r="G155" s="33"/>
+      <c r="G155" s="21"/>
       <c r="H155" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="156" customHeight="1" ht="18.75">
@@ -8937,7 +8935,7 @@
       <c r="D156" s="32"/>
       <c r="E156" s="2"/>
       <c r="F156" s="22"/>
-      <c r="G156" s="33"/>
+      <c r="G156" s="21"/>
       <c r="H156" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="157" customHeight="1" ht="18.75">
@@ -8947,7 +8945,7 @@
       <c r="D157" s="32"/>
       <c r="E157" s="2"/>
       <c r="F157" s="22"/>
-      <c r="G157" s="33"/>
+      <c r="G157" s="21"/>
       <c r="H157" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="158" customHeight="1" ht="18.75">
@@ -8957,7 +8955,7 @@
       <c r="D158" s="32"/>
       <c r="E158" s="2"/>
       <c r="F158" s="22"/>
-      <c r="G158" s="33"/>
+      <c r="G158" s="21"/>
       <c r="H158" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="159" customHeight="1" ht="18.75">
@@ -8967,7 +8965,7 @@
       <c r="D159" s="32"/>
       <c r="E159" s="2"/>
       <c r="F159" s="22"/>
-      <c r="G159" s="33"/>
+      <c r="G159" s="21"/>
       <c r="H159" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="160" customHeight="1" ht="18.75">
@@ -8977,7 +8975,7 @@
       <c r="D160" s="32"/>
       <c r="E160" s="2"/>
       <c r="F160" s="22"/>
-      <c r="G160" s="33"/>
+      <c r="G160" s="21"/>
       <c r="H160" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="18.75">
@@ -8987,7 +8985,7 @@
       <c r="D161" s="32"/>
       <c r="E161" s="2"/>
       <c r="F161" s="22"/>
-      <c r="G161" s="33"/>
+      <c r="G161" s="21"/>
       <c r="H161" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="18.75">
@@ -8997,7 +8995,7 @@
       <c r="D162" s="32"/>
       <c r="E162" s="2"/>
       <c r="F162" s="22"/>
-      <c r="G162" s="33"/>
+      <c r="G162" s="21"/>
       <c r="H162" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="18.75">
@@ -9007,7 +9005,7 @@
       <c r="D163" s="32"/>
       <c r="E163" s="2"/>
       <c r="F163" s="22"/>
-      <c r="G163" s="33"/>
+      <c r="G163" s="21"/>
       <c r="H163" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="18.75">
@@ -9017,7 +9015,7 @@
       <c r="D164" s="32"/>
       <c r="E164" s="2"/>
       <c r="F164" s="22"/>
-      <c r="G164" s="33"/>
+      <c r="G164" s="21"/>
       <c r="H164" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="18.75">
@@ -9027,7 +9025,7 @@
       <c r="D165" s="32"/>
       <c r="E165" s="2"/>
       <c r="F165" s="22"/>
-      <c r="G165" s="33"/>
+      <c r="G165" s="21"/>
       <c r="H165" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="18.75">
@@ -9037,7 +9035,7 @@
       <c r="D166" s="32"/>
       <c r="E166" s="2"/>
       <c r="F166" s="22"/>
-      <c r="G166" s="33"/>
+      <c r="G166" s="21"/>
       <c r="H166" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="18.75">
@@ -9047,7 +9045,7 @@
       <c r="D167" s="32"/>
       <c r="E167" s="2"/>
       <c r="F167" s="22"/>
-      <c r="G167" s="33"/>
+      <c r="G167" s="21"/>
       <c r="H167" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="18.75">
@@ -9057,7 +9055,7 @@
       <c r="D168" s="32"/>
       <c r="E168" s="2"/>
       <c r="F168" s="22"/>
-      <c r="G168" s="33"/>
+      <c r="G168" s="21"/>
       <c r="H168" s="2"/>
     </row>
   </sheetData>

</xml_diff>